<commit_message>
📊 RSI Report — 2026-05-28 [auto]
</commit_message>
<xml_diff>
--- a/output/RSI_Screener_2026-05-28.xlsx
+++ b/output/RSI_Screener_2026-05-28.xlsx
@@ -497,7 +497,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NSE500  |  RSI Screener  |  Run: 28-May-2026 08:23 IST  |  0 stocks matched</t>
+          <t>NSE500  |  RSI Screener  |  Run: 28-May-2026 08:50 IST  |  0 stocks matched</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MicroCap250  |  RSI Screener  |  Run: 28-May-2026 08:26 IST  |  0 stocks matched</t>
+          <t>MicroCap250  |  RSI Screener  |  Run: 28-May-2026 08:52 IST  |  0 stocks matched</t>
         </is>
       </c>
     </row>

</xml_diff>